<commit_message>
Pizza Sales Data Analysis (SQL) Group commit
</commit_message>
<xml_diff>
--- a/SQL_Projects/Pizza_Sales_Data_Analysis/2_Descriptive_Sales_Analysis/Assets/Descriptive_Sales_Analysis_Excel.xlsx
+++ b/SQL_Projects/Pizza_Sales_Data_Analysis/2_Descriptive_Sales_Analysis/Assets/Descriptive_Sales_Analysis_Excel.xlsx
@@ -39,36 +39,36 @@
     <sheet name="Top Years" sheetId="30" r:id="rId30"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Bottom 10 Names (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Bottom 10 Names (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bottom 10 Pizza IDs (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bottom 10 Pizza IDs (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bottom 10 Pizza Type IDs (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Bottom 10 Pizza Type IDs (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Top 10 Dates (C (D A))'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Top 10 Dates (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Top 10 Dates (T S (D A))'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Top 10 Dates (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Top 10 Names (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Top 10 Names (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Top 10 Order Hours (C (H A))'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'Top 10 Order Hours (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Top 10 Order Hours (T S (H A))'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Top 10 Order Hours (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Top 10 Order Times (C (T A))'!$A$3:$M$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Top 10 Order Times (C)'!$A$3:$M$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Top 10 Order Times (T S (T A))'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Top 10 Order Times (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Top 10 Pizza IDs (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Top 10 Pizza IDs (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Top 10 Pizza Type IDs (C)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Top 10 Pizza Type IDs (T S)'!$A$3:$M$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Top Categories (T S)'!$A$3:$M$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Top Days'!$A$3:$M$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Top Months'!$A$3:$M$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Top Quarters'!$A$3:$M$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Top Sizes (T S)'!$A$3:$M$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'Top Years'!$A$3:$M$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Bottom 10 Names (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Bottom 10 Names (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Bottom 10 Pizza IDs (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bottom 10 Pizza IDs (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Bottom 10 Pizza Type IDs (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Bottom 10 Pizza Type IDs (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Top 10 Dates (C (D A))'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Top 10 Dates (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Top 10 Dates (T S (D A))'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Top 10 Dates (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Top 10 Names (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Top 10 Names (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="25" hidden="1">'Top 10 Order Hours (C (H A))'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="24" hidden="1">'Top 10 Order Hours (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Top 10 Order Hours (T S (H A))'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Top 10 Order Hours (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Top 10 Order Times (C (T A))'!$A$3:$M$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Top 10 Order Times (C)'!$A$3:$M$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Top 10 Order Times (T S (T A))'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Top 10 Order Times (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Top 10 Pizza IDs (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Top 10 Pizza IDs (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Top 10 Pizza Type IDs (C)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Top 10 Pizza Type IDs (T S)'!$A$3:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Top Categories (T S)'!$A$3:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="26" hidden="1">'Top Days'!$A$3:$M$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'Top Months'!$A$3:$M$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="28" hidden="1">'Top Quarters'!$A$3:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Top Sizes (T S)'!$A$3:$M$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="29" hidden="1">'Top Years'!$A$3:$M$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2772,7 +2772,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3365,7 +3365,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -3958,7 +3958,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -4551,7 +4551,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -4862,7 +4862,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M6"/>
+  <autoFilter ref="A3:M7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -5220,7 +5220,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M7"/>
+  <autoFilter ref="A3:M8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -5813,7 +5813,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6406,7 +6406,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -6999,7 +6999,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -7592,7 +7592,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -8185,7 +8185,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -8778,7 +8778,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -9371,7 +9371,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -11750,7 +11750,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M50"/>
+  <autoFilter ref="A3:M51"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -14129,7 +14129,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M50"/>
+  <autoFilter ref="A3:M51"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -14722,7 +14722,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -15315,7 +15315,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -15908,7 +15908,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -16501,7 +16501,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -16953,7 +16953,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M9"/>
+  <autoFilter ref="A3:M10"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -17640,7 +17640,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M14"/>
+  <autoFilter ref="A3:M15"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -17950,7 +17950,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M6"/>
+  <autoFilter ref="A3:M7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -18543,7 +18543,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -18713,7 +18713,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M3"/>
+  <autoFilter ref="A3:M4"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -19306,7 +19306,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -19899,7 +19899,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -20492,7 +20492,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -21085,7 +21085,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -21678,7 +21678,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>
@@ -22271,7 +22271,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M12"/>
+  <autoFilter ref="A3:M13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>